<commit_message>
Optimize API to gemini-2.0-flash, use gemini-embedding-2 with 1024 dimensions, clean raw handover data, and update sync scripts
</commit_message>
<xml_diff>
--- a/data/01_NyAh-PhuDinh/Giá & Thanh toán/BÁO CÁO CƠ SỞ DỮ LIỆU TỔNG LỰC_ DỰ ÁN NY'AH PHÚ ĐỊNH.xlsx
+++ b/data/01_NyAh-PhuDinh/Giá & Thanh toán/BÁO CÁO CƠ SỞ DỮ LIỆU TỔNG LỰC_ DỰ ÁN NY'AH PHÚ ĐỊNH.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\QuangLêBáDuy\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nhadatcompany.sharepoint.com/sites/TeamMktg/Shared Documents/NPD mktg/mktg - private/03_Content/ChatBotData_Upload/01_NyAh-PhuDinh/Giá &amp; Thanh toán/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B75F365C-F455-4DDB-B3AE-FDF802A7F0B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{B75F365C-F455-4DDB-B3AE-FDF802A7F0B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3714954C-AF3A-44A5-9E44-77F3B855CB98}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="1042" yWindow="1042" windowWidth="14400" windowHeight="8183" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table 1" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,20 @@
     <sheet name="Table 3" sheetId="3" r:id="rId3"/>
     <sheet name="Table 4" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -1030,9 +1043,9 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:B75"/>
-  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="12.59765625" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" ht="12.75">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1040,7 +1053,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" ht="12.75">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -1048,7 +1061,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" ht="12.75">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -1056,7 +1069,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" ht="12.75">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -1064,7 +1077,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" ht="12.75">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
@@ -1072,7 +1085,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" ht="12.75">
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
@@ -1361,7 +1374,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="12.59765625" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
@@ -1446,7 +1459,11 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="12.59765625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col min="1" max="1" width="43.33203125" customWidth="1"/>
+    <col min="2" max="2" width="27.53125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
@@ -1602,7 +1619,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="12.59765625" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
@@ -1750,8 +1767,28 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Tài liệu" ma:contentTypeID="0x0101003421C2F09A4BEA46A5B5AE4284068530" ma:contentTypeVersion="19" ma:contentTypeDescription="Tạo tài liệu mới." ma:contentTypeScope="" ma:versionID="0105140007f2305d9417dfbf075ce41f">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="300fa37b-2a09-4011-a0db-c11ba6d392f7" xmlns:ns3="a16b777b-eb0b-4844-aa73-ac2af43907aa" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a71f74b658475c2068fd45b507226f2a" ns2:_="" ns3:_="">
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="a16b777b-eb0b-4844-aa73-ac2af43907aa" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="300fa37b-2a09-4011-a0db-c11ba6d392f7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003421C2F09A4BEA46A5B5AE4284068530" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a7d3c9354d74b04def7b88790286df27">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="300fa37b-2a09-4011-a0db-c11ba6d392f7" xmlns:ns3="a16b777b-eb0b-4844-aa73-ac2af43907aa" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8c0ff748245dfcf92ad532111eb0443c" ns2:_="" ns3:_="">
     <xsd:import namespace="300fa37b-2a09-4011-a0db-c11ba6d392f7"/>
     <xsd:import namespace="a16b777b-eb0b-4844-aa73-ac2af43907aa"/>
     <xsd:element name="properties">
@@ -1841,7 +1878,7 @@
         </xsd:restriction>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="21" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Thẻ Hình ảnh" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="dc0e7fee-77db-48dd-853a-28ca3f641761" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="21" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="dc0e7fee-77db-48dd-853a-28ca3f641761" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
       <xsd:complexType>
         <xsd:sequence>
           <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
@@ -1867,7 +1904,7 @@
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="a16b777b-eb0b-4844-aa73-ac2af43907aa" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="15" nillable="true" ma:displayName="Chia sẻ Với" ma:internalName="SharedWithUsers" ma:readOnly="true">
+    <xsd:element name="SharedWithUsers" ma:index="15" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
       <xsd:complexType>
         <xsd:complexContent>
           <xsd:extension base="dms:UserMulti">
@@ -1886,7 +1923,7 @@
         </xsd:complexContent>
       </xsd:complexType>
     </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="16" nillable="true" ma:displayName="Chia sẻ Có Chi tiết" ma:internalName="SharedWithDetails" ma:readOnly="true">
+    <xsd:element name="SharedWithDetails" ma:index="16" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note">
           <xsd:maxLength value="255"/>
@@ -1914,8 +1951,8 @@
         <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Loại Nội dung"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Tiêu đề"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
         <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
         <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
@@ -2004,34 +2041,25 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="a16b777b-eb0b-4844-aa73-ac2af43907aa" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="300fa37b-2a09-4011-a0db-c11ba6d392f7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2E356476-5B4A-46DA-BFD0-0A7FB683E199}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A92222AC-0296-49AE-9154-31A0C972EB7A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a16b777b-eb0b-4844-aa73-ac2af43907aa"/>
+    <ds:schemaRef ds:uri="300fa37b-2a09-4011-a0db-c11ba6d392f7"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{752C11FE-0148-45F2-A26D-EC899B6FFDEF}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{752C11FE-0148-45F2-A26D-EC899B6FFDEF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A92222AC-0296-49AE-9154-31A0C972EB7A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9B5A6D3-361C-48C1-9F4C-DA2C4ABE2D87}"/>
 </file>
</xml_diff>